<commit_message>
Fix Dish Index Excel export corruption by preserving template x14 validations.
Stop rewriting data validations in ExcelJS; merge template sheet footer back after export and expand T_DishIndex range.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/assets/dish-index-export-template.xlsx
+++ b/assets/dish-index-export-template.xlsx
@@ -9395,8 +9395,8 @@
 </file>
 
 <file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="23" xr:uid="{2E2E5F06-10C2-4E56-B83B-DE2900E8C30D}" name="T_DishIndex" displayName="T_DishIndex" ref="B2:BB12" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="B2:BB12" xr:uid="{2E2E5F06-10C2-4E56-B83B-DE2900E8C30D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="23" xr:uid="{2E2E5F06-10C2-4E56-B83B-DE2900E8C30D}" name="T_DishIndex" displayName="T_DishIndex" ref="B2:BB500" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="B2:BB500" xr:uid="{2E2E5F06-10C2-4E56-B83B-DE2900E8C30D}"/>
   <tableColumns count="53">
     <tableColumn id="1" xr3:uid="{B8CEDDF4-9174-4970-AF0A-EFE79D2BB723}" name="Schema Version"/>
     <tableColumn id="2" xr3:uid="{FA5E7AA9-454B-4D01-95CC-460E7207F005}" name="Dish Code"/>

</xml_diff>